<commit_message>
Auto: Add chapter "一盒餅乾" (book: 三上)
</commit_message>
<xml_diff>
--- a/content-pipeline/inputs/book04/b04_ch01_final.xlsx
+++ b/content-pipeline/inputs/book04/b04_ch01_final.xlsx
@@ -543,7 +543,7 @@
 莉文阿姨是個粗心的人，經常會做出一些令自己都哭笑不得的事情。以下是她給我講的一段有趣的經歷。
 一天，莉文阿姨在機場候機。為了打發時間，她買了一盒餅乾和一本書，然後找了一個座位，坐下來專心地看起書來。
 突然，她發現坐在身旁的一個男人伸出手抓起放在他倆中間的餅乾喫。莉文阿姨很喫驚，但她想也許那人是餓壞了，於是沒有說什麼，只是也從盒子裏抓起餅乾來喫。
-那個男人看到莉文阿姨喫餅乾，似乎也喫了一驚，但他也沒有出聲，只是對她友好地笑笑，繼續拿餅乾喫。當喫到最後一塊餅乾時，他不好意思地笑笑，把餅乾掰成兩半，一半給自己，一半遞給莉文。莉文阿姨接過半塊餅乾，心想：這個『飢餓的強盜』還不算太壞，居然平分了餅乾。
+那個男人看到莉文阿姨喫餅乾，似乎也喫了一驚，但他也沒有出聲，只是對她友好地笑笑，繼續拿餅乾喫。當喫到最後一塊餅乾時，他不好意思地笑笑，把餅乾掰成兩半，一半給自己，一半遞給莉文。莉文阿姨接過半塊餅乾，心想：這個「飢餓的強盜」還不算太壞，居然平分了餅乾。
 聽到登機通知後，莉文阿姨急忙把書塞進袋裏，拿起行李，直奔登機口。當她在飛機上坐好後，從袋裏掏出沒看完的書，準備繼續看時，突然愣住了，她這才發現，原來自己的那盒餅乾還原封不動地放在袋裏！剛才她喫的正是那個男人的餅乾。</t>
         </is>
       </c>
@@ -566,7 +566,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>don't know whether to laugh or cry</t>
+          <t>not know whether to laugh or cry</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>waiting for the flight</t>
+          <t>wait for the flight</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>very hungry</t>
+          <t>starved</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>speak</t>
+          <t>say anything</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>break in half</t>
+          <t>break into two halves</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>handed to</t>
+          <t>hand over to</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>boarding call</t>
+          <t>boarding announcement</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>rushed straight to</t>
+          <t>headed straight for</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,8 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>莉文阿姨是個粗心的人，經常會做出一些令自己都哭笑不得的事情。</t>
+          <t>三上 ：一盒餅乾 （第六頁）
+莉文阿姨是個粗心的人，經常會做出一些令自己都哭笑不得的事情。</t>
         </is>
       </c>
     </row>
@@ -920,7 +921,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>don't know whether to laugh or cry</t>
+          <t>not know whether to laugh or cry</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -930,7 +931,8 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>莉文阿姨是個粗心的人，經常會做出一些令自己都哭笑不得的事情。</t>
+          <t>三上 ：一盒餅乾 （第六頁）
+莉文阿姨是個粗心的人，經常會做出一些令自己都哭笑不得的事情。</t>
         </is>
       </c>
     </row>
@@ -964,7 +966,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>waiting for the flight</t>
+          <t>wait for the flight</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -996,7 +998,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>為了打發時間，她買了一盒餅乾和一本書。</t>
+          <t>為了打發時間，她買了一盒餅乾和一本書，然後找了一個座位，坐下來專心地看起書來。</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1020,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>她坐下來專心地看起書來。</t>
+          <t>為了打發時間，她買了一盒餅乾和一本書，然後找了一個座位，坐下來專心地看起書來。</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1042,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>她發現坐在身旁的一個男人抓起餅乾喫。</t>
+          <t>突然，她發現坐在身旁的一個男人伸出手抓起放在他倆中間的餅乾喫。</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1064,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>莉文阿姨很喫驚，但沒有說什麼。</t>
+          <t>莉文阿姨很喫驚，但她想也許那人是餓壞了，於是沒有說什麼，只是也從盒子裏抓起餅乾來喫。</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1076,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>very hungry</t>
+          <t>starved</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1084,7 +1086,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>她想也許那人是餓壞了。</t>
+          <t>莉文阿姨很喫驚，但她想也許那人是餓壞了，於是沒有說什麼，只是也從盒子裏抓起餅乾來喫。</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1098,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>speak</t>
+          <t>say anything</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1106,7 +1108,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>他沒有出聲，只是對她友好地笑笑。</t>
+          <t>那個男人看到莉文阿姨喫餅乾，似乎也喫了一驚，但他也沒有出聲，只是對她友好地笑笑，繼續拿餅乾喫。</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1130,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>他對她友好地笑笑，繼續拿餅乾喫。</t>
+          <t>那個男人看到莉文阿姨喫餅乾，似乎也喫了一驚，但他也沒有出聲，只是對她友好地笑笑，繼續拿餅乾喫。</t>
         </is>
       </c>
     </row>
@@ -1140,7 +1142,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>break in half</t>
+          <t>break into two halves</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1150,7 +1152,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>他把餅乾掰成兩半，一半給自己。</t>
+          <t>當喫到最後一塊餅乾時，他不好意思地笑笑，把餅乾掰成兩半，一半給自己，一半遞給莉文。</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1164,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>handed to</t>
+          <t>hand over to</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1172,7 +1174,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>他一半遞給莉文。</t>
+          <t>當喫到最後一塊餅乾時，他不好意思地笑笑，把餅乾掰成兩半，一半給自己，一半遞給莉文。</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1196,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>她心想這個『飢餓的強盜』還不算太壞。</t>
+          <t>莉文阿姨接過半塊餅乾，心想：這個「飢餓的強盜」還不算太壞，居然平分了餅乾。</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1218,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>她心想這個『飢餓的強盜』還不算太壞。</t>
+          <t>莉文阿姨接過半塊餅乾，心想：這個「飢餓的強盜」還不算太壞，居然平分了餅乾。</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1240,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>他居然平分了餅乾。</t>
+          <t>莉文阿姨接過半塊餅乾，心想：這個「飢餓的強盜」還不算太壞，居然平分了餅乾。</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1252,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>boarding call</t>
+          <t>boarding announcement</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1260,7 +1262,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>聽到登機通知後，她直奔登機口。</t>
+          <t>聽到登機通知後，莉文阿姨急忙把書塞進袋裏，拿起行李，直奔登機口。</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1284,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>莉文阿姨急忙把書塞進袋裏。</t>
+          <t>聽到登機通知後，莉文阿姨急忙把書塞進袋裏，拿起行李，直奔登機口。</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1306,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>她急忙把書塞進袋裏。</t>
+          <t>聽到登機通知後，莉文阿姨急忙把書塞進袋裏，拿起行李，直奔登機口。</t>
         </is>
       </c>
     </row>
@@ -1316,7 +1318,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>rushed straight to</t>
+          <t>headed straight for</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1326,7 +1328,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>她拿起行李，直奔登機口。</t>
+          <t>聽到登機通知後，莉文阿姨急忙把書塞進袋裏，拿起行李，直奔登機口。</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1350,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>她拿起行李，直奔登機口。</t>
+          <t>聽到登機通知後，莉文阿姨急忙把書塞進袋裏，拿起行李，直奔登機口。</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1372,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>她從袋裏掏出沒看完的書。</t>
+          <t>當她在飛機上坐好後，從袋裏掏出沒看完的書，準備繼續看時，突然愣住了，她這才發現，原來自己的那盒餅乾還原封不動地放在袋裏！</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1394,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>她突然愣住了，發現餅乾原封不動。</t>
+          <t>當她在飛機上坐好後，從袋裏掏出沒看完的書，準備繼續看時，突然愣住了，她這才發現，原來自己的那盒餅乾還原封不動地放在袋裏！</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1416,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>自己的那盒餅乾還原封不動地放在袋裏。</t>
+          <t>當她在飛機上坐好後，從袋裏掏出沒看完的書，準備繼續看時，突然愣住了，她這才發現，原來自己的那盒餅乾還原封不動地放在袋裏！</t>
         </is>
       </c>
     </row>

</xml_diff>